<commit_message>
bug fixed and updated data
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -9801,34 +9801,34 @@
       <c r="H189" s="8" t="inlineStr"/>
       <c r="I189" s="8" t="inlineStr"/>
       <c r="J189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="K189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="L189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="M189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="N189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="O189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="P189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="Q189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="R189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
       <c r="S189" s="8" t="n">
-        <v>72</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="190">
@@ -10205,34 +10205,34 @@
       <c r="H198" s="7" t="inlineStr"/>
       <c r="I198" s="7" t="inlineStr"/>
       <c r="J198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="K198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="L198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="M198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="N198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="O198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="P198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="Q198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="R198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="S198" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="199">
@@ -10557,34 +10557,34 @@
       <c r="H206" s="8" t="inlineStr"/>
       <c r="I206" s="8" t="inlineStr"/>
       <c r="J206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="K206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="L206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="M206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="N206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="O206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="P206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="Q206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="R206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="S206" s="8" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="207">
@@ -10909,34 +10909,34 @@
       <c r="H214" s="7" t="inlineStr"/>
       <c r="I214" s="7" t="inlineStr"/>
       <c r="J214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="K214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="L214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="M214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="N214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="O214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="P214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="Q214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="R214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
       <c r="S214" s="7" t="n">
-        <v>99</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="215">
@@ -15964,12 +15964,17 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>emi_n2o_p_x2x</t>
+          <t>sec_syngas</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -15981,24 +15986,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sec_lpg_orig</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>emi_ch4_f_x2x</t>
         </is>
       </c>
     </row>
@@ -16010,7 +16010,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>sec_methane</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -16027,7 +16027,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
+          <t>pri_coal</t>
         </is>
       </c>
     </row>
@@ -16039,7 +16039,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sec_heat_high</t>
+          <t>sec_diesel_fos_orig</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
+          <t>sec_kerosene_orig</t>
         </is>
       </c>
     </row>
@@ -16068,7 +16068,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
+          <t>sec_methane</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16080,7 +16085,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pri_deuterium</t>
+          <t>sec_lng_orig</t>
         </is>
       </c>
     </row>
@@ -16092,7 +16097,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>sec_heavy_fuel_oil_orig</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16104,12 +16114,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sec_ammonia</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>€/MWh</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
     </row>
@@ -16121,7 +16126,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>pri_coal</t>
+          <t>sec_naphtha_orig</t>
         </is>
       </c>
     </row>
@@ -16133,7 +16138,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>sec_lng</t>
         </is>
       </c>
     </row>
@@ -16145,7 +16150,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sec_ethanol</t>
+          <t>sec_diesel</t>
         </is>
       </c>
     </row>
@@ -16157,7 +16162,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
+          <t>pri_uran</t>
         </is>
       </c>
     </row>
@@ -16169,24 +16174,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_lpg</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>t/t</t>
+          <t>sec_cng</t>
         </is>
       </c>
     </row>
@@ -16198,7 +16198,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>sec_heat_low</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -16215,19 +16215,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>sec_gasoline_fos_orig</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sec_ethanol_orig</t>
+          <t>emi_co2_f_x2x</t>
         </is>
       </c>
     </row>
@@ -16239,7 +16244,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sec_lng_orig</t>
+          <t>sec_methanol</t>
         </is>
       </c>
     </row>
@@ -16251,48 +16256,48 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>emi_co2_p_x2x</t>
+          <t>sec_syngas_sr</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
+          <t>emi_n2o_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_air_bio</t>
         </is>
       </c>
     </row>
@@ -16304,12 +16309,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
     </row>
@@ -16321,7 +16321,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>sec_methane_orig</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16333,12 +16338,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>t/MWh</t>
+          <t>emi_ch4_p_x2x</t>
         </is>
       </c>
     </row>
@@ -16350,7 +16350,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
+          <t>sec_natural_gas_syn</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -16362,12 +16362,17 @@
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emi_co2_f_x2x</t>
+          <t>sec_heat_high</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16379,7 +16384,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_refinery_gas</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16391,12 +16401,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
     </row>
@@ -16408,12 +16413,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sec_biogas</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
     </row>
@@ -16425,7 +16425,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
+          <t>pri_deuterium</t>
         </is>
       </c>
     </row>
@@ -16437,24 +16437,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sec_elec</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sec_cng</t>
+          <t>emi_n2o_f_x2x</t>
         </is>
       </c>
     </row>
@@ -16466,7 +16461,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
+          <t>sec_biogas</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -16478,24 +16473,29 @@
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>emi_co2_neg_imp</t>
+          <t>pri_natural_gas</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>emi_ch4_p_x2x</t>
+          <t>sec_naphtha_fos_orig</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16507,19 +16507,29 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
+          <t>sec_ammonia</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>€/MWh</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_bio</t>
+          <t>sec_elec</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -16531,7 +16541,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_heavy_fuel_oil</t>
         </is>
       </c>
     </row>
@@ -16543,7 +16553,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -16555,17 +16565,17 @@
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>t/t</t>
         </is>
       </c>
     </row>
@@ -16577,24 +16587,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_ethanol</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_imp</t>
         </is>
       </c>
     </row>
@@ -16606,31 +16611,41 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
+          <t>sec_biokerosene_orig</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>emi_n2o_f_x2x</t>
+          <t>sec_lpg_orig</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>pri_uran</t>
+          <t>emi_co2_reusable</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>t/MWh</t>
         </is>
       </c>
     </row>
@@ -16642,7 +16657,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sec_lng</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
     </row>
@@ -16654,24 +16669,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>sec_refinery_gas</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sec_methanol</t>
+          <t>emi_co2_p_x2x</t>
         </is>
       </c>
     </row>
@@ -16683,12 +16693,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
     </row>
@@ -16700,7 +16705,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>sec_ethanol_orig</t>
         </is>
       </c>
     </row>
@@ -16712,7 +16717,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil_orig</t>
+          <t>pri_crude_oil</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -16729,7 +16734,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>sec_hydrogen_orig</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -16741,12 +16746,12 @@
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>emi_ch4_f_x2x</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
     </row>
@@ -16758,12 +16763,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
     </row>
@@ -16859,7 +16859,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Activity Unit</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -17291,7 +17291,7 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -17318,7 +17318,7 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -17345,7 +17345,7 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -17372,7 +17372,7 @@
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -17399,7 +17399,7 @@
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -17426,7 +17426,7 @@
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -17453,7 +17453,7 @@
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -17480,7 +17480,7 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -17507,7 +17507,7 @@
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -17534,7 +17534,7 @@
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -17561,7 +17561,7 @@
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -17588,7 +17588,7 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -17615,7 +17615,7 @@
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -17642,7 +17642,7 @@
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>IMP</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -17679,12 +17679,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -17731,6 +17731,11 @@
           <t>x2x_other_dac_ht_1</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>NO</t>
@@ -17748,6 +17753,11 @@
           <t>x2x_other_dac_lt_1</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>NO</t>
@@ -17794,12 +17804,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -17848,12 +17858,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -17902,12 +17912,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -17919,7 +17929,7 @@
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>STS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -17946,7 +17956,7 @@
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>STS</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -17973,7 +17983,7 @@
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>STS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -18000,7 +18010,7 @@
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>STS</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -18037,12 +18047,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -18224,6 +18234,11 @@
           <t>x2x_x2liquid_ft_1</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>NO</t>
@@ -18243,12 +18258,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -18270,12 +18285,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
+          <t>NRGI</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">

</xml_diff>

<commit_message>
comm grp bug fixes
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -503,7 +503,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -14139,7 +14139,11 @@
       </c>
       <c r="E280" s="7" t="inlineStr"/>
       <c r="F280" s="7" t="inlineStr"/>
-      <c r="G280" s="7" t="inlineStr"/>
+      <c r="G280" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H280" s="7" t="inlineStr"/>
       <c r="I280" s="7" t="inlineStr"/>
       <c r="J280" s="7" t="inlineStr"/>
@@ -14171,7 +14175,11 @@
           <t>sec_diesel_syn_orig</t>
         </is>
       </c>
-      <c r="G281" s="7" t="inlineStr"/>
+      <c r="G281" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H281" s="7" t="inlineStr"/>
       <c r="I281" s="7" t="inlineStr">
         <is>
@@ -14227,7 +14235,11 @@
           <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
-      <c r="G282" s="7" t="inlineStr"/>
+      <c r="G282" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H282" s="7" t="inlineStr"/>
       <c r="I282" s="7" t="inlineStr">
         <is>
@@ -14283,7 +14295,11 @@
           <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
-      <c r="G283" s="7" t="inlineStr"/>
+      <c r="G283" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H283" s="7" t="inlineStr"/>
       <c r="I283" s="7" t="inlineStr">
         <is>
@@ -14339,7 +14355,11 @@
           <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
-      <c r="G284" s="7" t="inlineStr"/>
+      <c r="G284" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H284" s="7" t="inlineStr"/>
       <c r="I284" s="7" t="inlineStr">
         <is>
@@ -14635,7 +14655,11 @@
           <t>sec_diesel_syn_orig</t>
         </is>
       </c>
-      <c r="G290" s="7" t="inlineStr"/>
+      <c r="G290" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H290" s="7" t="inlineStr"/>
       <c r="I290" s="7" t="inlineStr">
         <is>
@@ -14691,7 +14715,11 @@
           <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
-      <c r="G291" s="7" t="inlineStr"/>
+      <c r="G291" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H291" s="7" t="inlineStr"/>
       <c r="I291" s="7" t="inlineStr">
         <is>
@@ -14747,7 +14775,11 @@
           <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
-      <c r="G292" s="7" t="inlineStr"/>
+      <c r="G292" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H292" s="7" t="inlineStr"/>
       <c r="I292" s="7" t="inlineStr">
         <is>
@@ -14803,7 +14835,11 @@
           <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
-      <c r="G293" s="7" t="inlineStr"/>
+      <c r="G293" s="7" t="inlineStr">
+        <is>
+          <t>cg_d_g_k_n</t>
+        </is>
+      </c>
       <c r="H293" s="7" t="inlineStr"/>
       <c r="I293" s="7" t="inlineStr">
         <is>
@@ -15007,7 +15043,11 @@
       </c>
       <c r="E297" s="8" t="inlineStr"/>
       <c r="F297" s="8" t="inlineStr"/>
-      <c r="G297" s="8" t="inlineStr"/>
+      <c r="G297" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H297" s="8" t="inlineStr"/>
       <c r="I297" s="8" t="inlineStr"/>
       <c r="J297" s="8" t="n">
@@ -15059,7 +15099,11 @@
           <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
-      <c r="G298" s="8" t="inlineStr"/>
+      <c r="G298" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H298" s="8" t="inlineStr"/>
       <c r="I298" s="8" t="inlineStr">
         <is>
@@ -15115,7 +15159,11 @@
           <t>sec_diesel_fos_orig</t>
         </is>
       </c>
-      <c r="G299" s="8" t="inlineStr"/>
+      <c r="G299" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H299" s="8" t="inlineStr"/>
       <c r="I299" s="8" t="inlineStr">
         <is>
@@ -15171,7 +15219,11 @@
           <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
-      <c r="G300" s="8" t="inlineStr"/>
+      <c r="G300" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H300" s="8" t="inlineStr"/>
       <c r="I300" s="8" t="inlineStr">
         <is>
@@ -15227,7 +15279,11 @@
           <t>sec_lpg_orig</t>
         </is>
       </c>
-      <c r="G301" s="8" t="inlineStr"/>
+      <c r="G301" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H301" s="8" t="inlineStr"/>
       <c r="I301" s="8" t="inlineStr">
         <is>
@@ -15283,7 +15339,11 @@
           <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
-      <c r="G302" s="8" t="inlineStr"/>
+      <c r="G302" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H302" s="8" t="inlineStr"/>
       <c r="I302" s="8" t="inlineStr">
         <is>
@@ -15339,7 +15399,11 @@
           <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
-      <c r="G303" s="8" t="inlineStr"/>
+      <c r="G303" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H303" s="8" t="inlineStr"/>
       <c r="I303" s="8" t="inlineStr">
         <is>
@@ -15395,7 +15459,11 @@
           <t>sec_refinery_gas</t>
         </is>
       </c>
-      <c r="G304" s="8" t="inlineStr"/>
+      <c r="G304" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H304" s="8" t="inlineStr"/>
       <c r="I304" s="8" t="inlineStr">
         <is>
@@ -15691,7 +15759,11 @@
           <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
-      <c r="G310" s="8" t="inlineStr"/>
+      <c r="G310" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H310" s="8" t="inlineStr"/>
       <c r="I310" s="8" t="inlineStr">
         <is>
@@ -15747,7 +15819,11 @@
           <t>sec_diesel_fos_orig</t>
         </is>
       </c>
-      <c r="G311" s="8" t="inlineStr"/>
+      <c r="G311" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H311" s="8" t="inlineStr"/>
       <c r="I311" s="8" t="inlineStr">
         <is>
@@ -15803,7 +15879,11 @@
           <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
-      <c r="G312" s="8" t="inlineStr"/>
+      <c r="G312" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H312" s="8" t="inlineStr"/>
       <c r="I312" s="8" t="inlineStr">
         <is>
@@ -15859,7 +15939,11 @@
           <t>sec_lpg_orig</t>
         </is>
       </c>
-      <c r="G313" s="8" t="inlineStr"/>
+      <c r="G313" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H313" s="8" t="inlineStr"/>
       <c r="I313" s="8" t="inlineStr">
         <is>
@@ -15915,7 +15999,11 @@
           <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
-      <c r="G314" s="8" t="inlineStr"/>
+      <c r="G314" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H314" s="8" t="inlineStr"/>
       <c r="I314" s="8" t="inlineStr">
         <is>
@@ -15971,7 +16059,11 @@
           <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
-      <c r="G315" s="8" t="inlineStr"/>
+      <c r="G315" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H315" s="8" t="inlineStr"/>
       <c r="I315" s="8" t="inlineStr">
         <is>
@@ -16027,7 +16119,11 @@
           <t>sec_refinery_gas</t>
         </is>
       </c>
-      <c r="G316" s="8" t="inlineStr"/>
+      <c r="G316" s="8" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H316" s="8" t="inlineStr"/>
       <c r="I316" s="8" t="inlineStr">
         <is>
@@ -16231,7 +16327,11 @@
       </c>
       <c r="E320" s="7" t="inlineStr"/>
       <c r="F320" s="7" t="inlineStr"/>
-      <c r="G320" s="7" t="inlineStr"/>
+      <c r="G320" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H320" s="7" t="inlineStr"/>
       <c r="I320" s="7" t="inlineStr"/>
       <c r="J320" s="7" t="n">
@@ -16283,7 +16383,11 @@
           <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
-      <c r="G321" s="7" t="inlineStr"/>
+      <c r="G321" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H321" s="7" t="inlineStr"/>
       <c r="I321" s="7" t="inlineStr">
         <is>
@@ -16339,7 +16443,11 @@
           <t>sec_diesel_fos_orig</t>
         </is>
       </c>
-      <c r="G322" s="7" t="inlineStr"/>
+      <c r="G322" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H322" s="7" t="inlineStr"/>
       <c r="I322" s="7" t="inlineStr">
         <is>
@@ -16395,7 +16503,11 @@
           <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
-      <c r="G323" s="7" t="inlineStr"/>
+      <c r="G323" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H323" s="7" t="inlineStr"/>
       <c r="I323" s="7" t="inlineStr">
         <is>
@@ -16451,7 +16563,11 @@
           <t>sec_lpg_orig</t>
         </is>
       </c>
-      <c r="G324" s="7" t="inlineStr"/>
+      <c r="G324" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H324" s="7" t="inlineStr"/>
       <c r="I324" s="7" t="inlineStr">
         <is>
@@ -16507,7 +16623,11 @@
           <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
-      <c r="G325" s="7" t="inlineStr"/>
+      <c r="G325" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H325" s="7" t="inlineStr"/>
       <c r="I325" s="7" t="inlineStr">
         <is>
@@ -16563,7 +16683,11 @@
           <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
-      <c r="G326" s="7" t="inlineStr"/>
+      <c r="G326" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H326" s="7" t="inlineStr"/>
       <c r="I326" s="7" t="inlineStr">
         <is>
@@ -16619,7 +16743,11 @@
           <t>sec_refinery_gas</t>
         </is>
       </c>
-      <c r="G327" s="7" t="inlineStr"/>
+      <c r="G327" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H327" s="7" t="inlineStr"/>
       <c r="I327" s="7" t="inlineStr">
         <is>
@@ -16867,7 +16995,11 @@
           <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
-      <c r="G332" s="7" t="inlineStr"/>
+      <c r="G332" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H332" s="7" t="inlineStr"/>
       <c r="I332" s="7" t="inlineStr">
         <is>
@@ -16923,7 +17055,11 @@
           <t>sec_diesel_fos_orig</t>
         </is>
       </c>
-      <c r="G333" s="7" t="inlineStr"/>
+      <c r="G333" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H333" s="7" t="inlineStr"/>
       <c r="I333" s="7" t="inlineStr">
         <is>
@@ -16979,7 +17115,11 @@
           <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
-      <c r="G334" s="7" t="inlineStr"/>
+      <c r="G334" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H334" s="7" t="inlineStr"/>
       <c r="I334" s="7" t="inlineStr">
         <is>
@@ -17035,7 +17175,11 @@
           <t>sec_lpg_orig</t>
         </is>
       </c>
-      <c r="G335" s="7" t="inlineStr"/>
+      <c r="G335" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H335" s="7" t="inlineStr"/>
       <c r="I335" s="7" t="inlineStr">
         <is>
@@ -17091,7 +17235,11 @@
           <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
-      <c r="G336" s="7" t="inlineStr"/>
+      <c r="G336" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H336" s="7" t="inlineStr"/>
       <c r="I336" s="7" t="inlineStr">
         <is>
@@ -17147,7 +17295,11 @@
           <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
-      <c r="G337" s="7" t="inlineStr"/>
+      <c r="G337" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H337" s="7" t="inlineStr"/>
       <c r="I337" s="7" t="inlineStr">
         <is>
@@ -17203,7 +17355,11 @@
           <t>sec_refinery_gas</t>
         </is>
       </c>
-      <c r="G338" s="7" t="inlineStr"/>
+      <c r="G338" s="7" t="inlineStr">
+        <is>
+          <t>cg_g_d_k_l_n_h_r</t>
+        </is>
+      </c>
       <c r="H338" s="7" t="inlineStr"/>
       <c r="I338" s="7" t="inlineStr">
         <is>
@@ -18008,46 +18164,41 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_co2_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_ch4_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>emi_n2o_f_x2x</t>
+          <t>sec_kerosene_orig</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18059,7 +18210,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>sec_ethanol</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -18071,12 +18222,17 @@
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pri_uran</t>
+          <t>emi_co2_reusable</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>t</t>
         </is>
       </c>
     </row>
@@ -18088,7 +18244,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>sec_biogas</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -18105,12 +18261,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sec_methane</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
     </row>
@@ -18122,7 +18273,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>sec_methane_orig</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -18139,12 +18290,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_hydrogen_orig</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -18156,12 +18307,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
+          <t>sec_heat_low</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>MWh</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -18173,12 +18329,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_deuterium</t>
         </is>
       </c>
     </row>
@@ -18190,7 +18341,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -18219,29 +18370,29 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>emi_n2o_p_x2x</t>
+          <t>sec_naphtha_orig</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sec_refinery_gas</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_ch4_f_x2x</t>
         </is>
       </c>
     </row>
@@ -18253,7 +18404,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>sec_methanol</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -18270,7 +18421,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
+          <t>sec_kerosene_syn_orig</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18282,7 +18438,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil_orig</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -18299,7 +18455,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_biokerosene_orig</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -18316,12 +18472,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>pri_coal</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -18333,24 +18489,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>emi_co2_f_x2x</t>
+          <t>sec_kerosene</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18362,7 +18518,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
+          <t>sec_diesel</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -18379,7 +18535,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
+          <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -18396,7 +18552,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>sec_ethanol</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -18408,12 +18564,12 @@
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>emi_n2o_f_x2x</t>
         </is>
       </c>
     </row>
@@ -18425,7 +18581,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sec_lng_orig</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -18442,7 +18598,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>sec_ammonia</t>
+          <t>sec_lpg_orig</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -18454,12 +18610,17 @@
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>emi_ch4_f_x2x</t>
+          <t>sec_ammonia_orig</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18471,7 +18632,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
+          <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -18483,17 +18644,12 @@
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_co2_f_x2x</t>
         </is>
       </c>
     </row>
@@ -18505,7 +18661,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>pri_crude_oil</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -18522,17 +18678,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sec_elec</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>MWh</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -18544,17 +18695,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>sec_heat_high</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>MWh</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -18566,7 +18712,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_ethanol_orig</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -18583,7 +18729,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
+          <t>sec_syngas</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -18595,12 +18741,17 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>emi_co2_p_x2x</t>
+          <t>sec_natural_gas_syn</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18612,24 +18763,34 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>MWh</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>emi_co2_neg_imp</t>
+          <t>sec_heavy_fuel_oil</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18641,17 +18802,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>MWh</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -18663,12 +18819,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
+          <t>sec_heat_high</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>MWh</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -18680,7 +18841,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>sec_lng_orig</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -18697,29 +18858,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_uran</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>t</t>
         </is>
       </c>
     </row>
@@ -18731,12 +18887,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18748,7 +18904,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sec_methanol</t>
+          <t>sec_ammonia</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -18765,12 +18921,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>t</t>
+          <t>emi_co2_neg_imp</t>
         </is>
       </c>
     </row>
@@ -18782,7 +18933,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>pri_deuterium</t>
+          <t>sec_cng</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18794,7 +18950,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_biogas</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -18811,7 +18967,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sec_cng</t>
+          <t>sec_refinery_gas</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -18828,7 +18984,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -18840,41 +18996,51 @@
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>sec_lng</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>emi_ch4_p_x2x</t>
+          <t>pri_natural_gas</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_bio</t>
+          <t>sec_diesel_fos_orig</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18886,12 +19052,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sec_ethanol_orig</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -18903,7 +19069,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>pri_coal</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -18915,34 +19081,24 @@
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sec_lpg_orig</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_n2o_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_lng</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_co2_neg_air_bio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
act eff and process list bug fix
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -14458,36 +14458,16 @@
       <c r="G290" s="7" t="inlineStr"/>
       <c r="H290" s="7" t="inlineStr"/>
       <c r="I290" s="7" t="inlineStr"/>
-      <c r="J290" s="7" t="n">
-        <v>1.3677</v>
-      </c>
-      <c r="K290" s="7" t="n">
-        <v>1.3613</v>
-      </c>
-      <c r="L290" s="7" t="n">
-        <v>1.3548</v>
-      </c>
-      <c r="M290" s="7" t="n">
-        <v>1.3484</v>
-      </c>
-      <c r="N290" s="7" t="n">
-        <v>1.3377</v>
-      </c>
-      <c r="O290" s="7" t="n">
-        <v>1.3269</v>
-      </c>
-      <c r="P290" s="7" t="n">
-        <v>1.3162</v>
-      </c>
-      <c r="Q290" s="7" t="n">
-        <v>1.3055</v>
-      </c>
-      <c r="R290" s="7" t="n">
-        <v>1.3055</v>
-      </c>
-      <c r="S290" s="7" t="n">
-        <v>1.3055</v>
-      </c>
+      <c r="J290" s="7" t="inlineStr"/>
+      <c r="K290" s="7" t="inlineStr"/>
+      <c r="L290" s="7" t="inlineStr"/>
+      <c r="M290" s="7" t="inlineStr"/>
+      <c r="N290" s="7" t="inlineStr"/>
+      <c r="O290" s="7" t="inlineStr"/>
+      <c r="P290" s="7" t="inlineStr"/>
+      <c r="Q290" s="7" t="inlineStr"/>
+      <c r="R290" s="7" t="inlineStr"/>
+      <c r="S290" s="7" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="B291" s="7" t="inlineStr">
@@ -14510,36 +14490,16 @@
       <c r="G291" s="7" t="inlineStr"/>
       <c r="H291" s="7" t="inlineStr"/>
       <c r="I291" s="7" t="inlineStr"/>
-      <c r="J291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="L291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="M291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="N291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="O291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="Q291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="R291" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="S291" s="7" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="J291" s="7" t="inlineStr"/>
+      <c r="K291" s="7" t="inlineStr"/>
+      <c r="L291" s="7" t="inlineStr"/>
+      <c r="M291" s="7" t="inlineStr"/>
+      <c r="N291" s="7" t="inlineStr"/>
+      <c r="O291" s="7" t="inlineStr"/>
+      <c r="P291" s="7" t="inlineStr"/>
+      <c r="Q291" s="7" t="inlineStr"/>
+      <c r="R291" s="7" t="inlineStr"/>
+      <c r="S291" s="7" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="B292" s="7" t="inlineStr">
@@ -15362,36 +15322,16 @@
       <c r="G307" s="8" t="inlineStr"/>
       <c r="H307" s="8" t="inlineStr"/>
       <c r="I307" s="8" t="inlineStr"/>
-      <c r="J307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="K307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="L307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="M307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="N307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="O307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="P307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="Q307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="R307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="S307" s="8" t="n">
-        <v>1.1038</v>
-      </c>
+      <c r="J307" s="8" t="inlineStr"/>
+      <c r="K307" s="8" t="inlineStr"/>
+      <c r="L307" s="8" t="inlineStr"/>
+      <c r="M307" s="8" t="inlineStr"/>
+      <c r="N307" s="8" t="inlineStr"/>
+      <c r="O307" s="8" t="inlineStr"/>
+      <c r="P307" s="8" t="inlineStr"/>
+      <c r="Q307" s="8" t="inlineStr"/>
+      <c r="R307" s="8" t="inlineStr"/>
+      <c r="S307" s="8" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="B308" s="8" t="inlineStr">
@@ -16646,36 +16586,16 @@
       <c r="G330" s="7" t="inlineStr"/>
       <c r="H330" s="7" t="inlineStr"/>
       <c r="I330" s="7" t="inlineStr"/>
-      <c r="J330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="K330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="L330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="M330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="N330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="O330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="P330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="Q330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="R330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
-      <c r="S330" s="7" t="n">
-        <v>1.1038</v>
-      </c>
+      <c r="J330" s="7" t="inlineStr"/>
+      <c r="K330" s="7" t="inlineStr"/>
+      <c r="L330" s="7" t="inlineStr"/>
+      <c r="M330" s="7" t="inlineStr"/>
+      <c r="N330" s="7" t="inlineStr"/>
+      <c r="O330" s="7" t="inlineStr"/>
+      <c r="P330" s="7" t="inlineStr"/>
+      <c r="Q330" s="7" t="inlineStr"/>
+      <c r="R330" s="7" t="inlineStr"/>
+      <c r="S330" s="7" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="B331" s="7" t="inlineStr">
@@ -18585,7 +18505,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_ethanol_orig</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -18602,7 +18522,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -18619,58 +18539,48 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pri_biomass_pellets_pp</t>
+          <t>sec_naphtha_orig</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_co2_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_n2o_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_co2_f_x2x</t>
         </is>
       </c>
     </row>
@@ -18682,7 +18592,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pri_uran</t>
+          <t>pri_deuterium</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18604,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>pri_coal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18706,7 +18621,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -18723,7 +18638,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sec_methanol</t>
+          <t>sec_syngas</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -18735,12 +18650,22 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>emi_n2o_f_x2x</t>
+          <t>sec_heat_low</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -18752,7 +18677,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>sec_biogas</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -18769,7 +18694,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>pri_waste_municipal_bio</t>
+          <t>sec_biokerosene_orig</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18781,12 +18711,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -18798,7 +18733,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>emi_ch4_f_x2x</t>
+          <t>emi_co2_neg_air_bio</t>
         </is>
       </c>
     </row>
@@ -18810,12 +18745,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_uran</t>
         </is>
       </c>
     </row>
@@ -18827,17 +18757,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>MWh</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -18849,7 +18774,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_lng_orig</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -18861,12 +18786,12 @@
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pri_deuterium</t>
+          <t>emi_ch4_p_x2x</t>
         </is>
       </c>
     </row>
@@ -18878,12 +18803,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil_orig</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_waste_municipal_bio</t>
         </is>
       </c>
     </row>
@@ -18895,12 +18815,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sec_refinery_gas</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -18912,12 +18832,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -18929,24 +18849,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_waste_animal</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>emi_co2_neg_imp</t>
+          <t>pri_crude_oil</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18878,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sec_ammonia</t>
+          <t>sec_diesel</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -18975,7 +18895,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>sec_natural_gas_syn</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -18987,17 +18907,12 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_ch4_f_x2x</t>
         </is>
       </c>
     </row>
@@ -19009,7 +18924,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_cng</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -19026,7 +18941,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -19038,24 +18953,34 @@
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_bio</t>
+          <t>sec_heavy_fuel_oil</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>pri_waste_animal</t>
+          <t>emi_co2_neg_air_dacc</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>t</t>
         </is>
       </c>
     </row>
@@ -19067,7 +18992,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>pri_coal</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -19079,12 +19004,17 @@
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>emi_n2o_p_x2x</t>
+          <t>sec_refinery_gas</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -19096,7 +19026,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>sec_lpg_orig</t>
+          <t>sec_methanol</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -19113,7 +19043,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -19130,41 +19060,36 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_biomass_straw_bales_pr</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_n2o_f_x2x</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>emi_co2_p_x2x</t>
+          <t>sec_kerosene_syn_orig</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -19176,19 +19101,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>pri_biomass_straw_bales_pr</t>
+          <t>sec_lng_orig</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>emi_co2_f_x2x</t>
+          <t>sec_heat_high</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -19200,29 +19140,29 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
+          <t>pri_natural_gas</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sec_methane</t>
+          <t>emi_co2_reusable</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>t</t>
         </is>
       </c>
     </row>
@@ -19234,7 +19174,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>sec_kerosene_orig</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -19246,17 +19186,17 @@
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
+          <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -19268,17 +19208,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_heat_high</t>
+          <t>sec_lpg_orig</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>MWh</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -19290,7 +19225,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sec_ethanol_orig</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -19302,12 +19237,17 @@
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>emi_ch4_p_x2x</t>
+          <t>sec_gasoline_fos_orig</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -19319,7 +19259,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -19336,7 +19276,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_ethanol</t>
+          <t>sec_lng</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -19353,12 +19293,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>pri_biomass_pellets_pp</t>
         </is>
       </c>
     </row>
@@ -19370,7 +19305,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -19387,17 +19322,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sec_elec</t>
+          <t>sec_hydrogen_orig</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MWh</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -19409,7 +19339,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sec_lng</t>
+          <t>sec_diesel_fos_orig</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -19426,7 +19356,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>sec_methane_orig</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -19443,7 +19373,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_biogas</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -19455,17 +19385,12 @@
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sec_cng</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>emi_co2_neg_imp</t>
         </is>
       </c>
     </row>
@@ -19477,7 +19402,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -19494,12 +19419,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
     </row>
@@ -19511,24 +19431,29 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
+          <t>sec_ammonia</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>MWh</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -19540,7 +19465,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>sec_ethanol</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -19557,12 +19482,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>MWh</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
     </row>
@@ -19695,7 +19615,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -19722,7 +19642,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -19749,7 +19669,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -19776,7 +19696,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -19803,7 +19723,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -19830,7 +19750,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -19857,7 +19777,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -19884,7 +19804,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -19911,7 +19831,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -19938,7 +19858,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -19965,7 +19885,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -19992,7 +19912,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -20019,7 +19939,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -20046,7 +19966,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -20073,7 +19993,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -20100,7 +20020,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -20127,7 +20047,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -20154,7 +20074,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -20181,7 +20101,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -20235,7 +20155,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -20262,7 +20182,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -20289,7 +20209,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -20316,7 +20236,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -20343,7 +20263,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -20370,7 +20290,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -20397,7 +20317,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -20424,7 +20344,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -20478,7 +20398,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -20505,7 +20425,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -20532,7 +20452,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>t</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -20559,7 +20479,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>t</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -20586,7 +20506,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -20613,7 +20533,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -20640,7 +20560,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -20667,7 +20587,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -20694,7 +20614,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -20721,7 +20641,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -20748,7 +20668,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -20775,7 +20695,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -20802,7 +20722,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -20829,7 +20749,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -20856,7 +20776,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -20883,7 +20803,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -20910,7 +20830,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -20937,7 +20857,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -20964,7 +20884,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -20991,7 +20911,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -21018,7 +20938,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -21045,7 +20965,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -21072,7 +20992,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -21126,7 +21046,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -21153,7 +21073,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -21207,7 +21127,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -21234,7 +21154,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">

</xml_diff>

<commit_message>
update _soec_ and _coel_ primary_cg to sec_elec
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -19863,7 +19863,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
+          <t>sec_lng</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -19880,12 +19880,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pri_waste_municipal_bio</t>
+          <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -19897,7 +19897,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil_orig</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -19926,17 +19926,17 @@
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
+          <t>sec_lpg_orig</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>t/MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -19948,7 +19948,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -19965,7 +19965,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sec_ammonia</t>
+          <t>sec_diesel_fos_orig</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -19982,7 +19982,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
+          <t>pri_natural_gas</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -19999,7 +19999,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pri_deuterium</t>
+          <t>sec_methane_orig</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20011,7 +20016,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
+          <t>sec_kerosene_orig</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -20028,7 +20033,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_biokerosene_orig</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -20040,17 +20045,12 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_n2o_f_x2x</t>
         </is>
       </c>
     </row>
@@ -20062,7 +20062,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sec_biogas</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -20079,17 +20079,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sec_elec</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -20101,29 +20096,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>t/t</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20135,7 +20135,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
+          <t>sec_ammonia</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -20147,17 +20147,12 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_ethanol</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_imp</t>
         </is>
       </c>
     </row>
@@ -20169,70 +20164,80 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>sec_methane</t>
+          <t>pri_waste_animal</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ/PJ</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>pri_biomass_straw_bales_pr</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>t/t</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_air_bio</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>emi_co2_p_x2x</t>
+          <t>sec_heat_high</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>emi_co2_neg_imp</t>
+          <t>pri_crude_oil</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20244,7 +20249,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>sec_refinery_gas</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -20283,12 +20288,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>pri_waste_municipal_bio</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ/PJ</t>
         </is>
       </c>
     </row>
@@ -20300,7 +20305,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>sec_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -20312,12 +20317,17 @@
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>emi_n2o_p_x2x</t>
+          <t>sec_natural_gas_syn</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20329,7 +20339,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>sec_cng</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -20341,12 +20351,17 @@
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emi_n2o_f_x2x</t>
+          <t>sec_hydrogen</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20358,7 +20373,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -20375,12 +20390,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_deuterium</t>
         </is>
       </c>
     </row>
@@ -20392,7 +20402,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -20409,7 +20419,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>pri_coal</t>
+          <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -20421,17 +20431,12 @@
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_n2o_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20443,7 +20448,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>pri_biomass_pellets_pp</t>
+          <t>pri_biomass_straw_bales_pr</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -20455,22 +20460,17 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sec_heat_high</t>
+          <t>emi_co2_reusable</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>t/MWh</t>
         </is>
       </c>
     </row>
@@ -20482,7 +20482,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sec_lng</t>
+          <t>sec_ethanol_orig</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -20499,7 +20499,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
+          <t>sec_syngas</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -20516,7 +20516,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
+          <t>pri_coal</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -20528,53 +20528,58 @@
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_f_x2x</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>emi_co2_f_x2x</t>
+          <t>sec_lng_orig</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>pri_uran</t>
+          <t>emi_ch4_f_x2x</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>emi_ch4_f_x2x</t>
+          <t>sec_naphtha_fos_orig</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20586,7 +20591,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -20603,7 +20608,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
+          <t>sec_diesel</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -20620,7 +20625,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>sec_naphtha_orig</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -20632,17 +20637,12 @@
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>sec_methanol</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20654,7 +20654,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_ethanol_orig</t>
+          <t>sec_biogas</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -20666,17 +20666,12 @@
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sec_refinery_gas</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_ch4_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20688,7 +20683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>pri_waste_animal</t>
+          <t>pri_biomass_pellets_pp</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -20705,7 +20700,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
+          <t>sec_ethanol</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -20717,12 +20712,17 @@
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>emi_ch4_p_x2x</t>
+          <t>sec_naphtha</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20734,12 +20734,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_uran</t>
         </is>
       </c>
     </row>
@@ -20751,7 +20746,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sec_lpg_orig</t>
+          <t>sec_methanol</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -20768,7 +20763,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -20785,7 +20780,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -20802,7 +20797,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_lng_orig</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -20819,7 +20814,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -20836,7 +20831,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>sec_cng</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -20848,12 +20843,17 @@
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_bio</t>
+          <t>sec_diesel_orig</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20865,7 +20865,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>sec_hydrogen_orig</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -22034,7 +22034,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>NRGI</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -22223,7 +22223,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>NRGI</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">

</xml_diff>

<commit_message>
update NRGI (input based) process ACT_EFF= conversion_factor_input (primary comm)
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S398"/>
+  <dimension ref="A1:S382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1" customWidth="1" min="1" max="1"/>
@@ -15089,34 +15089,34 @@
       <c r="H309" s="7" t="inlineStr"/>
       <c r="I309" s="7" t="inlineStr"/>
       <c r="J309" s="7" t="n">
-        <v>0.7311544929443592</v>
+        <v>1.3677</v>
       </c>
       <c r="K309" s="7" t="n">
-        <v>0.7345919341805627</v>
+        <v>1.3613</v>
       </c>
       <c r="L309" s="7" t="n">
-        <v>0.7381163271331562</v>
+        <v>1.3548</v>
       </c>
       <c r="M309" s="7" t="n">
-        <v>0.7416196974191634</v>
+        <v>1.3484</v>
       </c>
       <c r="N309" s="7" t="n">
-        <v>0.7475517679599313</v>
+        <v>1.3377</v>
       </c>
       <c r="O309" s="7" t="n">
-        <v>0.7536362951239732</v>
+        <v>1.3269</v>
       </c>
       <c r="P309" s="7" t="n">
-        <v>0.759762953958365</v>
+        <v>1.3162</v>
       </c>
       <c r="Q309" s="7" t="n">
-        <v>0.7659900421294522</v>
+        <v>1.3055</v>
       </c>
       <c r="R309" s="7" t="n">
-        <v>0.7659900421294522</v>
+        <v>1.3055</v>
       </c>
       <c r="S309" s="7" t="n">
-        <v>0.7659900421294522</v>
+        <v>1.3055</v>
       </c>
     </row>
     <row r="310">
@@ -16027,34 +16027,34 @@
       <c r="H327" s="8" t="inlineStr"/>
       <c r="I327" s="8" t="inlineStr"/>
       <c r="J327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="K327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="L327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="M327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="N327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="O327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="P327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="Q327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="R327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="S327" s="8" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
     </row>
     <row r="328">
@@ -17291,34 +17291,34 @@
       <c r="H350" s="7" t="inlineStr"/>
       <c r="I350" s="7" t="inlineStr"/>
       <c r="J350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="K350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="L350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="M350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="N350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="O350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="P350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="Q350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="R350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
       <c r="S350" s="7" t="n">
-        <v>0.9059612248595761</v>
+        <v>1.1038</v>
       </c>
     </row>
     <row r="351">
@@ -19032,810 +19032,6 @@
         <v>1</v>
       </c>
       <c r="S382" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="383">
-      <c r="B383" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biokerosene</t>
-        </is>
-      </c>
-      <c r="C383" s="8" t="inlineStr"/>
-      <c r="D383" s="8" t="inlineStr">
-        <is>
-          <t>ACT_COST</t>
-        </is>
-      </c>
-      <c r="E383" s="8" t="inlineStr"/>
-      <c r="F383" s="8" t="inlineStr"/>
-      <c r="G383" s="8" t="inlineStr"/>
-      <c r="H383" s="8" t="inlineStr"/>
-      <c r="I383" s="8" t="inlineStr"/>
-      <c r="J383" s="8" t="n">
-        <v>32.05555555555556</v>
-      </c>
-      <c r="K383" s="8" t="n">
-        <v>30.38888888888889</v>
-      </c>
-      <c r="L383" s="8" t="n">
-        <v>28.69444444444445</v>
-      </c>
-      <c r="M383" s="8" t="n">
-        <v>27.02777777777778</v>
-      </c>
-      <c r="N383" s="8" t="n">
-        <v>26.36111111111111</v>
-      </c>
-      <c r="O383" s="8" t="n">
-        <v>25.69444444444445</v>
-      </c>
-      <c r="P383" s="8" t="n">
-        <v>25.30555555555555</v>
-      </c>
-      <c r="Q383" s="8" t="n">
-        <v>24.88888888888889</v>
-      </c>
-      <c r="R383" s="8" t="n">
-        <v>24.88888888888889</v>
-      </c>
-      <c r="S383" s="8" t="n">
-        <v>24.88888888888889</v>
-      </c>
-    </row>
-    <row r="384">
-      <c r="B384" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biokerosene</t>
-        </is>
-      </c>
-      <c r="C384" s="8" t="inlineStr"/>
-      <c r="D384" s="8" t="inlineStr">
-        <is>
-          <t>CAP2ACT</t>
-        </is>
-      </c>
-      <c r="E384" s="8" t="inlineStr"/>
-      <c r="F384" s="8" t="inlineStr"/>
-      <c r="G384" s="8" t="inlineStr"/>
-      <c r="H384" s="8" t="inlineStr"/>
-      <c r="I384" s="8" t="inlineStr"/>
-      <c r="J384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R384" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S384" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="385">
-      <c r="B385" s="7" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_oref_1</t>
-        </is>
-      </c>
-      <c r="C385" s="7" t="inlineStr"/>
-      <c r="D385" s="7" t="inlineStr">
-        <is>
-          <t>FLO_SHAR</t>
-        </is>
-      </c>
-      <c r="E385" s="7" t="inlineStr"/>
-      <c r="F385" s="7" t="inlineStr">
-        <is>
-          <t>sec_refinery_gas</t>
-        </is>
-      </c>
-      <c r="G385" s="7" t="inlineStr">
-        <is>
-          <t>cg_g_d_k_l_n_h_r</t>
-        </is>
-      </c>
-      <c r="H385" s="7" t="inlineStr"/>
-      <c r="I385" s="7" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="J385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="K385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="L385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="N385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="O385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="P385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="Q385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="R385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="S385" s="7" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="386">
-      <c r="B386" s="7" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_oref_1</t>
-        </is>
-      </c>
-      <c r="C386" s="7" t="inlineStr"/>
-      <c r="D386" s="7" t="inlineStr">
-        <is>
-          <t>CAP2ACT</t>
-        </is>
-      </c>
-      <c r="E386" s="7" t="inlineStr"/>
-      <c r="F386" s="7" t="inlineStr"/>
-      <c r="G386" s="7" t="inlineStr"/>
-      <c r="H386" s="7" t="inlineStr"/>
-      <c r="I386" s="7" t="inlineStr"/>
-      <c r="J386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="K386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="L386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="M386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="N386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="O386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="P386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="Q386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="R386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-      <c r="S386" s="7" t="n">
-        <v>31.536</v>
-      </c>
-    </row>
-    <row r="387">
-      <c r="B387" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biodiesel</t>
-        </is>
-      </c>
-      <c r="C387" s="8" t="inlineStr"/>
-      <c r="D387" s="8" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="E387" s="8" t="inlineStr"/>
-      <c r="F387" s="8" t="inlineStr">
-        <is>
-          <t>sec_biodiesel_orig</t>
-        </is>
-      </c>
-      <c r="G387" s="8" t="inlineStr"/>
-      <c r="H387" s="8" t="inlineStr"/>
-      <c r="I387" s="8" t="inlineStr"/>
-      <c r="J387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R387" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S387" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="388">
-      <c r="B388" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biodiesel</t>
-        </is>
-      </c>
-      <c r="C388" s="8" t="inlineStr"/>
-      <c r="D388" s="8" t="inlineStr">
-        <is>
-          <t>NCAP_BND</t>
-        </is>
-      </c>
-      <c r="E388" s="8" t="inlineStr"/>
-      <c r="F388" s="8" t="inlineStr"/>
-      <c r="G388" s="8" t="inlineStr"/>
-      <c r="H388" s="8" t="inlineStr"/>
-      <c r="I388" s="8" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="J388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="K388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="L388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="M388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="N388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="O388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="P388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="Q388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="R388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-      <c r="S388" s="8" t="n">
-        <v>3.581178</v>
-      </c>
-    </row>
-    <row r="389">
-      <c r="B389" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biodiesel</t>
-        </is>
-      </c>
-      <c r="C389" s="8" t="inlineStr"/>
-      <c r="D389" s="8" t="inlineStr">
-        <is>
-          <t>ACT_COST</t>
-        </is>
-      </c>
-      <c r="E389" s="8" t="inlineStr"/>
-      <c r="F389" s="8" t="inlineStr"/>
-      <c r="G389" s="8" t="inlineStr"/>
-      <c r="H389" s="8" t="inlineStr"/>
-      <c r="I389" s="8" t="inlineStr"/>
-      <c r="J389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="K389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="L389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="M389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="N389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="O389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="P389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="Q389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="R389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-      <c r="S389" s="8" t="n">
-        <v>24.36111111111111</v>
-      </c>
-    </row>
-    <row r="390">
-      <c r="B390" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biodiesel</t>
-        </is>
-      </c>
-      <c r="C390" s="8" t="inlineStr"/>
-      <c r="D390" s="8" t="inlineStr">
-        <is>
-          <t>CAP2ACT</t>
-        </is>
-      </c>
-      <c r="E390" s="8" t="inlineStr"/>
-      <c r="F390" s="8" t="inlineStr"/>
-      <c r="G390" s="8" t="inlineStr"/>
-      <c r="H390" s="8" t="inlineStr"/>
-      <c r="I390" s="8" t="inlineStr"/>
-      <c r="J390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R390" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S390" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="391">
-      <c r="B391" s="7" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_bioethanol</t>
-        </is>
-      </c>
-      <c r="C391" s="7" t="inlineStr"/>
-      <c r="D391" s="7" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="E391" s="7" t="inlineStr"/>
-      <c r="F391" s="7" t="inlineStr">
-        <is>
-          <t>sec_ethanol_orig</t>
-        </is>
-      </c>
-      <c r="G391" s="7" t="inlineStr"/>
-      <c r="H391" s="7" t="inlineStr"/>
-      <c r="I391" s="7" t="inlineStr"/>
-      <c r="J391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="P391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="R391" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="S391" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="392">
-      <c r="B392" s="7" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_bioethanol</t>
-        </is>
-      </c>
-      <c r="C392" s="7" t="inlineStr"/>
-      <c r="D392" s="7" t="inlineStr">
-        <is>
-          <t>NCAP_BND</t>
-        </is>
-      </c>
-      <c r="E392" s="7" t="inlineStr"/>
-      <c r="F392" s="7" t="inlineStr"/>
-      <c r="G392" s="7" t="inlineStr"/>
-      <c r="H392" s="7" t="inlineStr"/>
-      <c r="I392" s="7" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="J392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="K392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="L392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="M392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="N392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="O392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="P392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="Q392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="R392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-      <c r="S392" s="7" t="n">
-        <v>0.412228</v>
-      </c>
-    </row>
-    <row r="393">
-      <c r="B393" s="7" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_bioethanol</t>
-        </is>
-      </c>
-      <c r="C393" s="7" t="inlineStr"/>
-      <c r="D393" s="7" t="inlineStr">
-        <is>
-          <t>ACT_COST</t>
-        </is>
-      </c>
-      <c r="E393" s="7" t="inlineStr"/>
-      <c r="F393" s="7" t="inlineStr"/>
-      <c r="G393" s="7" t="inlineStr"/>
-      <c r="H393" s="7" t="inlineStr"/>
-      <c r="I393" s="7" t="inlineStr"/>
-      <c r="J393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="K393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="L393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="M393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="N393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="O393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="P393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="Q393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="R393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-      <c r="S393" s="7" t="n">
-        <v>21.05555555555556</v>
-      </c>
-    </row>
-    <row r="394">
-      <c r="B394" s="7" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_bioethanol</t>
-        </is>
-      </c>
-      <c r="C394" s="7" t="inlineStr"/>
-      <c r="D394" s="7" t="inlineStr">
-        <is>
-          <t>CAP2ACT</t>
-        </is>
-      </c>
-      <c r="E394" s="7" t="inlineStr"/>
-      <c r="F394" s="7" t="inlineStr"/>
-      <c r="G394" s="7" t="inlineStr"/>
-      <c r="H394" s="7" t="inlineStr"/>
-      <c r="I394" s="7" t="inlineStr"/>
-      <c r="J394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="P394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="R394" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="S394" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="395">
-      <c r="B395" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biokerosene</t>
-        </is>
-      </c>
-      <c r="C395" s="8" t="inlineStr"/>
-      <c r="D395" s="8" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="E395" s="8" t="inlineStr"/>
-      <c r="F395" s="8" t="inlineStr">
-        <is>
-          <t>sec_biokerosene_orig</t>
-        </is>
-      </c>
-      <c r="G395" s="8" t="inlineStr"/>
-      <c r="H395" s="8" t="inlineStr"/>
-      <c r="I395" s="8" t="inlineStr"/>
-      <c r="J395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R395" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S395" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="396">
-      <c r="B396" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biokerosene</t>
-        </is>
-      </c>
-      <c r="C396" s="8" t="inlineStr"/>
-      <c r="D396" s="8" t="inlineStr">
-        <is>
-          <t>NCAP_BND</t>
-        </is>
-      </c>
-      <c r="E396" s="8" t="inlineStr"/>
-      <c r="F396" s="8" t="inlineStr"/>
-      <c r="G396" s="8" t="inlineStr"/>
-      <c r="H396" s="8" t="inlineStr"/>
-      <c r="I396" s="8" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="J396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="K396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="L396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="M396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="N396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="O396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="P396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="Q396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="R396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-      <c r="S396" s="8" t="n">
-        <v>1.506849</v>
-      </c>
-    </row>
-    <row r="397">
-      <c r="B397" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biokerosene</t>
-        </is>
-      </c>
-      <c r="C397" s="8" t="inlineStr"/>
-      <c r="D397" s="8" t="inlineStr">
-        <is>
-          <t>ACT_COST</t>
-        </is>
-      </c>
-      <c r="E397" s="8" t="inlineStr"/>
-      <c r="F397" s="8" t="inlineStr"/>
-      <c r="G397" s="8" t="inlineStr"/>
-      <c r="H397" s="8" t="inlineStr"/>
-      <c r="I397" s="8" t="inlineStr"/>
-      <c r="J397" s="8" t="n">
-        <v>32.05555555555556</v>
-      </c>
-      <c r="K397" s="8" t="n">
-        <v>30.38888888888889</v>
-      </c>
-      <c r="L397" s="8" t="n">
-        <v>28.69444444444445</v>
-      </c>
-      <c r="M397" s="8" t="n">
-        <v>27.02777777777778</v>
-      </c>
-      <c r="N397" s="8" t="n">
-        <v>26.36111111111111</v>
-      </c>
-      <c r="O397" s="8" t="n">
-        <v>25.69444444444445</v>
-      </c>
-      <c r="P397" s="8" t="n">
-        <v>25.30555555555555</v>
-      </c>
-      <c r="Q397" s="8" t="n">
-        <v>24.88888888888889</v>
-      </c>
-      <c r="R397" s="8" t="n">
-        <v>24.88888888888889</v>
-      </c>
-      <c r="S397" s="8" t="n">
-        <v>24.88888888888889</v>
-      </c>
-    </row>
-    <row r="398">
-      <c r="B398" s="8" t="inlineStr">
-        <is>
-          <t>x2x_x2liquid_source_biokerosene</t>
-        </is>
-      </c>
-      <c r="C398" s="8" t="inlineStr"/>
-      <c r="D398" s="8" t="inlineStr">
-        <is>
-          <t>CAP2ACT</t>
-        </is>
-      </c>
-      <c r="E398" s="8" t="inlineStr"/>
-      <c r="F398" s="8" t="inlineStr"/>
-      <c r="G398" s="8" t="inlineStr"/>
-      <c r="H398" s="8" t="inlineStr"/>
-      <c r="I398" s="8" t="inlineStr"/>
-      <c r="J398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R398" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S398" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -19958,22 +19154,12 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sec_elec</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>emi_n2o_f_x2x</t>
         </is>
       </c>
     </row>
@@ -19985,7 +19171,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sec_biogas</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20002,36 +19188,41 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_waste_animal</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>emi_ch4_p_x2x</t>
+          <t>pri_natural_gas</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>emi_co2_f_x2x</t>
+          <t>sec_gasoline_syn_orig</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20043,7 +19234,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -20060,36 +19251,46 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pri_deuterium</t>
+          <t>sec_heat_high</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_refinery_gas</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_air_bio</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>emi_co2_p_x2x</t>
+          <t>sec_lpg_orig</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20101,29 +19302,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sec_methane</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_deuterium</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_n2o_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20135,7 +19326,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -20152,17 +19343,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
+          <t>sec_ethanol</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -20174,7 +19360,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
+          <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -20191,7 +19377,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sec_lng_orig</t>
+          <t>sec_methanol</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -20208,12 +19394,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_waste_municipal_bio</t>
         </is>
       </c>
     </row>
@@ -20225,7 +19406,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sec_ethanol</t>
+          <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -20237,17 +19418,12 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_ch4_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20259,7 +19435,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>sec_syngas</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -20276,7 +19452,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
+          <t>sec_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -20293,7 +19469,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil_orig</t>
+          <t>sec_refinery_gas</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -20310,12 +19486,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_biomass_pellets_pp</t>
         </is>
       </c>
     </row>
@@ -20327,7 +19498,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -20356,29 +19527,29 @@
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_ch4_f_x2x</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>emi_ch4_f_x2x</t>
+          <t>sec_biokerosene_orig</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20390,7 +19561,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -20407,41 +19578,46 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>pri_waste_animal</t>
+          <t>sec_lng</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
+          <t>sec_diesel</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>t/MWh</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emi_n2o_f_x2x</t>
+          <t>sec_kerosene_orig</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20453,7 +19629,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
+          <t>sec_diesel_fos_orig</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -20470,7 +19646,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -20487,7 +19663,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
+          <t>sec_lng_orig</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -20504,12 +19680,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>pri_biomass_pellets_pp</t>
+          <t>sec_methane_orig</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20521,29 +19697,29 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sec_ethanol_orig</t>
+          <t>sec_heat_low</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20555,12 +19731,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>pri_biomass_straw_bales_pr</t>
+          <t>sec_hydrogen_orig</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20572,7 +19748,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_naphtha_orig</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -20584,29 +19760,29 @@
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_bio</t>
+          <t>pri_coal</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sec_ammonia</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_f_x2x</t>
         </is>
       </c>
     </row>
@@ -20618,12 +19794,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sec_methanol</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -20635,7 +19816,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sec_lng</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -20652,7 +19833,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>pri_coal</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -20669,7 +19850,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -20686,24 +19867,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_uran</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>emi_co2_neg_imp</t>
+          <t>sec_ammonia</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20715,12 +19896,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_biomass_straw_bales_pr</t>
         </is>
       </c>
     </row>
@@ -20732,7 +19908,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>pri_uran</t>
+          <t>pri_crude_oil</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20744,17 +19925,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_heat_high</t>
+          <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -20766,7 +19942,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -20778,12 +19954,17 @@
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>emi_n2o_p_x2x</t>
+          <t>sec_biogas</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20795,7 +19976,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -20812,7 +19993,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -20829,7 +20010,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -20846,29 +20027,29 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>pri_waste_municipal_bio</t>
+          <t>sec_cng</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sec_cng</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>t/t</t>
         </is>
       </c>
     </row>
@@ -20880,7 +20061,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -20897,7 +20078,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -20909,51 +20090,46 @@
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>sec_lpg_orig</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_imp</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>sec_natural_gas_syn</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>t/t</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>emi_co2_reusable</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>t/MWh</t>
         </is>
       </c>
     </row>
@@ -20965,7 +20141,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>sec_ethanol_orig</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">

</xml_diff>

<commit_message>
update output and configuration files; add unit conversion in emission factors
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -7260,36 +7260,16 @@
       <c r="G141" s="8" t="inlineStr"/>
       <c r="H141" s="8" t="inlineStr"/>
       <c r="I141" s="8" t="inlineStr"/>
-      <c r="J141" s="8" t="n">
-        <v>0.001296</v>
-      </c>
-      <c r="K141" s="8" t="n">
-        <v>0.001296</v>
-      </c>
-      <c r="L141" s="8" t="n">
-        <v>0.0051444</v>
-      </c>
-      <c r="M141" s="8" t="n">
-        <v>0.004986</v>
-      </c>
-      <c r="N141" s="8" t="n">
-        <v>0.004986</v>
-      </c>
-      <c r="O141" s="8" t="n">
-        <v>0.004986</v>
-      </c>
-      <c r="P141" s="8" t="n">
-        <v>0.0048636</v>
-      </c>
-      <c r="Q141" s="8" t="n">
-        <v>0.00408996</v>
-      </c>
-      <c r="R141" s="8" t="n">
-        <v>0.00408996</v>
-      </c>
-      <c r="S141" s="8" t="n">
-        <v>0.00408996</v>
-      </c>
+      <c r="J141" s="8" t="inlineStr"/>
+      <c r="K141" s="8" t="inlineStr"/>
+      <c r="L141" s="8" t="inlineStr"/>
+      <c r="M141" s="8" t="inlineStr"/>
+      <c r="N141" s="8" t="inlineStr"/>
+      <c r="O141" s="8" t="inlineStr"/>
+      <c r="P141" s="8" t="inlineStr"/>
+      <c r="Q141" s="8" t="inlineStr"/>
+      <c r="R141" s="8" t="inlineStr"/>
+      <c r="S141" s="8" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="B142" s="8" t="inlineStr">
@@ -7312,36 +7292,16 @@
       <c r="G142" s="8" t="inlineStr"/>
       <c r="H142" s="8" t="inlineStr"/>
       <c r="I142" s="8" t="inlineStr"/>
-      <c r="J142" s="8" t="n">
-        <v>0.004428</v>
-      </c>
-      <c r="K142" s="8" t="n">
-        <v>0.004428</v>
-      </c>
-      <c r="L142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R142" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="S142" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="J142" s="8" t="inlineStr"/>
+      <c r="K142" s="8" t="inlineStr"/>
+      <c r="L142" s="8" t="inlineStr"/>
+      <c r="M142" s="8" t="inlineStr"/>
+      <c r="N142" s="8" t="inlineStr"/>
+      <c r="O142" s="8" t="inlineStr"/>
+      <c r="P142" s="8" t="inlineStr"/>
+      <c r="Q142" s="8" t="inlineStr"/>
+      <c r="R142" s="8" t="inlineStr"/>
+      <c r="S142" s="8" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="B143" s="8" t="inlineStr">
@@ -7694,36 +7654,16 @@
       <c r="G150" s="7" t="inlineStr"/>
       <c r="H150" s="7" t="inlineStr"/>
       <c r="I150" s="7" t="inlineStr"/>
-      <c r="J150" s="7" t="n">
-        <v>0.0009</v>
-      </c>
-      <c r="K150" s="7" t="n">
-        <v>0.000864</v>
-      </c>
-      <c r="L150" s="7" t="n">
-        <v>0.0008370000000000001</v>
-      </c>
-      <c r="M150" s="7" t="n">
-        <v>0.00081</v>
-      </c>
-      <c r="N150" s="7" t="n">
-        <v>0.0007704</v>
-      </c>
-      <c r="O150" s="7" t="n">
-        <v>0.0007308</v>
-      </c>
-      <c r="P150" s="7" t="n">
-        <v>0.000693</v>
-      </c>
-      <c r="Q150" s="7" t="n">
-        <v>0.00057582</v>
-      </c>
-      <c r="R150" s="7" t="n">
-        <v>0.00057582</v>
-      </c>
-      <c r="S150" s="7" t="n">
-        <v>0.00057582</v>
-      </c>
+      <c r="J150" s="7" t="inlineStr"/>
+      <c r="K150" s="7" t="inlineStr"/>
+      <c r="L150" s="7" t="inlineStr"/>
+      <c r="M150" s="7" t="inlineStr"/>
+      <c r="N150" s="7" t="inlineStr"/>
+      <c r="O150" s="7" t="inlineStr"/>
+      <c r="P150" s="7" t="inlineStr"/>
+      <c r="Q150" s="7" t="inlineStr"/>
+      <c r="R150" s="7" t="inlineStr"/>
+      <c r="S150" s="7" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="B151" s="7" t="inlineStr">
@@ -7746,36 +7686,16 @@
       <c r="G151" s="7" t="inlineStr"/>
       <c r="H151" s="7" t="inlineStr"/>
       <c r="I151" s="7" t="inlineStr"/>
-      <c r="J151" s="7" t="n">
-        <v>0.0063</v>
-      </c>
-      <c r="K151" s="7" t="n">
-        <v>0.005939999999999999</v>
-      </c>
-      <c r="L151" s="7" t="n">
-        <v>0.00567</v>
-      </c>
-      <c r="M151" s="7" t="n">
-        <v>0.0054</v>
-      </c>
-      <c r="N151" s="7" t="n">
-        <v>0.0050148</v>
-      </c>
-      <c r="O151" s="7" t="n">
-        <v>0.0046296</v>
-      </c>
-      <c r="P151" s="7" t="n">
-        <v>0.0042984</v>
-      </c>
-      <c r="Q151" s="7" t="n">
-        <v>0.00353772</v>
-      </c>
-      <c r="R151" s="7" t="n">
-        <v>0.00353772</v>
-      </c>
-      <c r="S151" s="7" t="n">
-        <v>0.00353772</v>
-      </c>
+      <c r="J151" s="7" t="inlineStr"/>
+      <c r="K151" s="7" t="inlineStr"/>
+      <c r="L151" s="7" t="inlineStr"/>
+      <c r="M151" s="7" t="inlineStr"/>
+      <c r="N151" s="7" t="inlineStr"/>
+      <c r="O151" s="7" t="inlineStr"/>
+      <c r="P151" s="7" t="inlineStr"/>
+      <c r="Q151" s="7" t="inlineStr"/>
+      <c r="R151" s="7" t="inlineStr"/>
+      <c r="S151" s="7" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="B152" s="7" t="inlineStr">
@@ -20187,7 +20107,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -20204,7 +20124,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>pri_crude_oil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20221,29 +20141,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sec_cng</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>pri_uran</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>t/t</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20255,7 +20170,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sec_lng_orig</t>
+          <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -20272,7 +20187,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sec_biogas</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -20289,7 +20204,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
+          <t>pri_natural_gas</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -20306,7 +20221,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_methanol</t>
+          <t>sec_natural_gas_syn</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -20323,7 +20238,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sec_lpg_orig</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -20340,7 +20255,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>pri_coal</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -20352,53 +20267,63 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>emi_co2_p_x2x</t>
+          <t>sec_hydrogen_orig</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>emi_n2o_p_x2x</t>
+          <t>pri_waste_animal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PJ/PJ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>emi_ch4_f_x2x</t>
+          <t>sec_syngas</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>t/MWh</t>
+          <t>emi_ch4_f_x2x</t>
         </is>
       </c>
     </row>
@@ -20410,7 +20335,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
+          <t>pri_coal</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -20427,7 +20352,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
+          <t>sec_lpg_orig</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -20439,12 +20364,17 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_bio</t>
+          <t>sec_diesel_fos_orig</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20456,12 +20386,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
+          <t>sec_heat_low</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -20473,12 +20408,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pri_bio_pellet_pp</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>PJ/PJ</t>
+          <t>pri_deuterium</t>
         </is>
       </c>
     </row>
@@ -20490,17 +20420,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sec_heat_high</t>
+          <t>sec_lng</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -20512,24 +20437,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>emi_n2o_f_x2x</t>
+          <t>emi_co2_p_x2x</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil_orig</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_n2o_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20541,12 +20461,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>pri_waste_animal</t>
+          <t>sec_ethanol_orig</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20558,7 +20478,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -20575,7 +20495,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>pri_uran</t>
+          <t>sec_naphtha_syn_orig</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20587,24 +20512,29 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pri_deuterium</t>
+          <t>sec_cng</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pri_waste_mbio</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>t/t</t>
         </is>
       </c>
     </row>
@@ -20616,7 +20546,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
+          <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -20633,7 +20563,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>sec_ethanol</t>
+          <t>sec_kerosene_orig</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -20650,12 +20580,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -20667,7 +20602,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
+          <t>sec_lng_orig</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -20684,7 +20619,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
+          <t>sec_biogas</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -20701,7 +20636,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
+          <t>sec_methane_orig</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -20713,17 +20648,12 @@
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_ch4_p_x2x</t>
         </is>
       </c>
     </row>
@@ -20735,7 +20665,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>sec_methanol</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -20752,7 +20682,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>sec_naphtha_orig</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -20769,7 +20699,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -20786,7 +20716,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sec_refinery_gas</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -20803,7 +20733,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -20820,7 +20750,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_ethanol</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -20837,17 +20767,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sec_elec</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -20859,7 +20784,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sec_hydrogen_orig</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -20871,17 +20796,12 @@
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_f_x2x</t>
         </is>
       </c>
     </row>
@@ -20893,12 +20813,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>pri_bio_straw</t>
+          <t>sec_biokerosene_orig</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>MWh/MWh</t>
         </is>
       </c>
     </row>
@@ -20910,7 +20830,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_lng</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -20922,12 +20842,17 @@
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>emi_co2_f_x2x</t>
+          <t>pri_waste_mbio</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PJ/PJ</t>
         </is>
       </c>
     </row>
@@ -20939,7 +20864,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -20951,34 +20876,24 @@
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>sec_methane</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_co2_neg_imp</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>MWh/MWh</t>
+          <t>emi_n2o_f_x2x</t>
         </is>
       </c>
     </row>
@@ -20990,7 +20905,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -21007,12 +20922,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>sec_ethanol_orig</t>
+          <t>sec_heat_high</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -21024,7 +20944,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -21036,12 +20956,17 @@
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>emi_ch4_p_x2x</t>
+          <t>pri_bio_straw</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>PJ/PJ</t>
         </is>
       </c>
     </row>
@@ -21053,17 +20978,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sec_heat_low</t>
+          <t>sec_ammonia</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>MWh/MWh</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -21075,7 +20995,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -21092,7 +21012,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_diesel</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -21104,17 +21024,17 @@
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>emi_co2_reusable</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>t/MWh</t>
         </is>
       </c>
     </row>
@@ -21126,7 +21046,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_ammonia</t>
+          <t>sec_heavy_fuel_oil_orig</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -21143,7 +21063,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>sec_refinery_gas</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -21160,7 +21080,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>emi_co2_neg_imp</t>
+          <t>emi_co2_neg_air_bio</t>
         </is>
       </c>
     </row>
@@ -21172,7 +21092,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
+          <t>sec_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -21189,12 +21109,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>pri_bio_pellet_pp</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ/PJ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update tcap and tact cols
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_x2x.xlsx
+++ b/output_data/vt_DE_x2x.xlsx
@@ -7260,16 +7260,36 @@
       <c r="G141" s="8" t="inlineStr"/>
       <c r="H141" s="8" t="inlineStr"/>
       <c r="I141" s="8" t="inlineStr"/>
-      <c r="J141" s="8" t="inlineStr"/>
-      <c r="K141" s="8" t="inlineStr"/>
-      <c r="L141" s="8" t="inlineStr"/>
-      <c r="M141" s="8" t="inlineStr"/>
-      <c r="N141" s="8" t="inlineStr"/>
-      <c r="O141" s="8" t="inlineStr"/>
-      <c r="P141" s="8" t="inlineStr"/>
-      <c r="Q141" s="8" t="inlineStr"/>
-      <c r="R141" s="8" t="inlineStr"/>
-      <c r="S141" s="8" t="inlineStr"/>
+      <c r="J141" s="8" t="n">
+        <v>0.001296</v>
+      </c>
+      <c r="K141" s="8" t="n">
+        <v>0.001296</v>
+      </c>
+      <c r="L141" s="8" t="n">
+        <v>0.0051444</v>
+      </c>
+      <c r="M141" s="8" t="n">
+        <v>0.004986</v>
+      </c>
+      <c r="N141" s="8" t="n">
+        <v>0.004986</v>
+      </c>
+      <c r="O141" s="8" t="n">
+        <v>0.004986</v>
+      </c>
+      <c r="P141" s="8" t="n">
+        <v>0.0048636</v>
+      </c>
+      <c r="Q141" s="8" t="n">
+        <v>0.00408996</v>
+      </c>
+      <c r="R141" s="8" t="n">
+        <v>0.00408996</v>
+      </c>
+      <c r="S141" s="8" t="n">
+        <v>0.00408996</v>
+      </c>
     </row>
     <row r="142">
       <c r="B142" s="8" t="inlineStr">
@@ -7292,16 +7312,36 @@
       <c r="G142" s="8" t="inlineStr"/>
       <c r="H142" s="8" t="inlineStr"/>
       <c r="I142" s="8" t="inlineStr"/>
-      <c r="J142" s="8" t="inlineStr"/>
-      <c r="K142" s="8" t="inlineStr"/>
-      <c r="L142" s="8" t="inlineStr"/>
-      <c r="M142" s="8" t="inlineStr"/>
-      <c r="N142" s="8" t="inlineStr"/>
-      <c r="O142" s="8" t="inlineStr"/>
-      <c r="P142" s="8" t="inlineStr"/>
-      <c r="Q142" s="8" t="inlineStr"/>
-      <c r="R142" s="8" t="inlineStr"/>
-      <c r="S142" s="8" t="inlineStr"/>
+      <c r="J142" s="8" t="n">
+        <v>0.004428</v>
+      </c>
+      <c r="K142" s="8" t="n">
+        <v>0.004428</v>
+      </c>
+      <c r="L142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S142" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="B143" s="8" t="inlineStr">
@@ -7654,16 +7694,36 @@
       <c r="G150" s="7" t="inlineStr"/>
       <c r="H150" s="7" t="inlineStr"/>
       <c r="I150" s="7" t="inlineStr"/>
-      <c r="J150" s="7" t="inlineStr"/>
-      <c r="K150" s="7" t="inlineStr"/>
-      <c r="L150" s="7" t="inlineStr"/>
-      <c r="M150" s="7" t="inlineStr"/>
-      <c r="N150" s="7" t="inlineStr"/>
-      <c r="O150" s="7" t="inlineStr"/>
-      <c r="P150" s="7" t="inlineStr"/>
-      <c r="Q150" s="7" t="inlineStr"/>
-      <c r="R150" s="7" t="inlineStr"/>
-      <c r="S150" s="7" t="inlineStr"/>
+      <c r="J150" s="7" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="K150" s="7" t="n">
+        <v>0.000864</v>
+      </c>
+      <c r="L150" s="7" t="n">
+        <v>0.0008370000000000001</v>
+      </c>
+      <c r="M150" s="7" t="n">
+        <v>0.00081</v>
+      </c>
+      <c r="N150" s="7" t="n">
+        <v>0.0007704</v>
+      </c>
+      <c r="O150" s="7" t="n">
+        <v>0.0007308</v>
+      </c>
+      <c r="P150" s="7" t="n">
+        <v>0.000693</v>
+      </c>
+      <c r="Q150" s="7" t="n">
+        <v>0.00057582</v>
+      </c>
+      <c r="R150" s="7" t="n">
+        <v>0.00057582</v>
+      </c>
+      <c r="S150" s="7" t="n">
+        <v>0.00057582</v>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="7" t="inlineStr">
@@ -7686,16 +7746,36 @@
       <c r="G151" s="7" t="inlineStr"/>
       <c r="H151" s="7" t="inlineStr"/>
       <c r="I151" s="7" t="inlineStr"/>
-      <c r="J151" s="7" t="inlineStr"/>
-      <c r="K151" s="7" t="inlineStr"/>
-      <c r="L151" s="7" t="inlineStr"/>
-      <c r="M151" s="7" t="inlineStr"/>
-      <c r="N151" s="7" t="inlineStr"/>
-      <c r="O151" s="7" t="inlineStr"/>
-      <c r="P151" s="7" t="inlineStr"/>
-      <c r="Q151" s="7" t="inlineStr"/>
-      <c r="R151" s="7" t="inlineStr"/>
-      <c r="S151" s="7" t="inlineStr"/>
+      <c r="J151" s="7" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="K151" s="7" t="n">
+        <v>0.005939999999999999</v>
+      </c>
+      <c r="L151" s="7" t="n">
+        <v>0.00567</v>
+      </c>
+      <c r="M151" s="7" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="N151" s="7" t="n">
+        <v>0.0050148</v>
+      </c>
+      <c r="O151" s="7" t="n">
+        <v>0.0046296</v>
+      </c>
+      <c r="P151" s="7" t="n">
+        <v>0.0042984</v>
+      </c>
+      <c r="Q151" s="7" t="n">
+        <v>0.00353772</v>
+      </c>
+      <c r="R151" s="7" t="n">
+        <v>0.00353772</v>
+      </c>
+      <c r="S151" s="7" t="n">
+        <v>0.00353772</v>
+      </c>
     </row>
     <row r="152">
       <c r="B152" s="7" t="inlineStr">
@@ -21213,11 +21293,7 @@
           <t>notFound</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Capacity Unit</t>
-        </is>
-      </c>
+      <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Timeslice Operational Level</t>
@@ -21247,7 +21323,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -21274,7 +21355,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -21301,7 +21387,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -21328,7 +21419,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -21355,7 +21451,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -21382,7 +21483,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -21409,7 +21515,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -21436,7 +21547,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -21463,7 +21579,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -21490,7 +21611,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -21517,7 +21643,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -21544,7 +21675,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -21571,7 +21707,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -21598,9 +21739,10 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>NRGO</t>
@@ -21625,9 +21767,10 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>NRGO</t>
@@ -21652,7 +21795,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -21679,7 +21827,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -21706,7 +21859,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -21733,7 +21891,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -21763,6 +21926,11 @@
           <t>notFound</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>pri_deuterium</t>
@@ -21787,7 +21955,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -21814,7 +21987,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -21841,7 +22019,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -21868,7 +22051,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -21895,7 +22083,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -21922,7 +22115,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -21949,7 +22147,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -21976,7 +22179,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -22006,6 +22214,11 @@
           <t>notFound</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>pri_uran</t>
@@ -22030,9 +22243,10 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>NRGI</t>
@@ -22057,9 +22271,10 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>sec_cng</t>
@@ -22084,9 +22299,10 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>t/t</t>
-        </is>
-      </c>
+          <t>kt</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>emi_co2_neg_air_dacc</t>
@@ -22111,9 +22327,10 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>t/t</t>
-        </is>
-      </c>
+          <t>kt</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>emi_co2_neg_air_dacc</t>
@@ -22138,9 +22355,10 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>sec_lng_orig</t>
@@ -22165,9 +22383,10 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>NRGI</t>
@@ -22192,9 +22411,10 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>sec_natural_gas_syn</t>
@@ -22219,9 +22439,10 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>NRGI</t>
@@ -22246,9 +22467,10 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>sec_natural_gas_syn</t>
@@ -22273,9 +22495,10 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>sec_elec</t>
@@ -22300,7 +22523,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -22327,7 +22555,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -22354,7 +22587,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -22381,7 +22619,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -22408,9 +22651,10 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>sec_biogas</t>
@@ -22435,9 +22679,10 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>sec_biogas</t>
@@ -22462,9 +22707,10 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>sec_elec</t>
@@ -22489,9 +22735,10 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>sec_hydrogen_orig</t>
@@ -22516,9 +22763,10 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>sec_syngas</t>
@@ -22543,9 +22791,10 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>sec_syngas_sr</t>
@@ -22570,9 +22819,10 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>sec_syngas_sr</t>
@@ -22597,9 +22847,10 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>sec_hydrogen_orig</t>
@@ -22624,9 +22875,10 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>sec_hydrogen_orig</t>
@@ -22654,6 +22906,7 @@
           <t>notFound</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>sec_syngas</t>
@@ -22678,9 +22931,10 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>NRGI</t>
@@ -22705,9 +22959,10 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>NRGI</t>
@@ -22732,9 +22987,10 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>sec_biodiesel_orig</t>
@@ -22759,9 +23015,10 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>sec_ethanol_orig</t>
@@ -22786,9 +23043,10 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>MWh/MWh</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>sec_biokerosene_orig</t>

</xml_diff>